<commit_message>
chore(excel): sync monsters.xlsx 从 json（含 DASHER）
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/excel/monsters.xlsx
+++ b/config/excel/monsters.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC15"/>
+  <dimension ref="A1:AC16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1958,6 +1958,99 @@
       </c>
       <c r="AC15" t="inlineStr"/>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>DASHER</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>冲刺怪</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>10</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" t="n">
+        <v>8</v>
+      </c>
+      <c r="J16" t="n">
+        <v>70</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>#8B0000</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="M16" t="n">
+        <v>1</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" t="n">
+        <v>0</v>
+      </c>
+      <c r="T16" t="n">
+        <v>3</v>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>Bat</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>Bat</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr"/>
+      <c r="X16" t="inlineStr"/>
+      <c r="Y16" t="inlineStr"/>
+      <c r="Z16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC16" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(excel): sync monsters/stages xlsx（含 TELEPORTER）
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/excel/monsters.xlsx
+++ b/config/excel/monsters.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC16"/>
+  <dimension ref="A1:AC17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2051,6 +2051,103 @@
       </c>
       <c r="AC16" t="inlineStr"/>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TELEPORTER</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" t="n">
+        <v>6</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>瞬移怪</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>80</v>
+      </c>
+      <c r="F17" t="n">
+        <v>2</v>
+      </c>
+      <c r="G17" t="n">
+        <v>12</v>
+      </c>
+      <c r="H17" t="n">
+        <v>2</v>
+      </c>
+      <c r="I17" t="n">
+        <v>12</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>#5a3a7a</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" t="n">
+        <v>320</v>
+      </c>
+      <c r="O17" t="n">
+        <v>140</v>
+      </c>
+      <c r="P17" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" t="n">
+        <v>0</v>
+      </c>
+      <c r="T17" t="n">
+        <v>3</v>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>Necromancer</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>Necromancer</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr"/>
+      <c r="X17" t="inlineStr"/>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>enemy_teleport_bolt</t>
+        </is>
+      </c>
+      <c r="Z17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC17" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>